<commit_message>
Add Q1 2026 P&L data, resolve Citrin March P&L items, add First Principles doc
</commit_message>
<xml_diff>
--- a/Datapath 2025 P&L to EBITDA.xlsx
+++ b/Datapath 2025 P&L to EBITDA.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="103">
   <si>
     <t xml:space="preserve">Datapath, Inc.</t>
   </si>
@@ -31,7 +31,7 @@
     <t xml:space="preserve">Profit &amp; Loss Statement - Monthly Detail Through EBITDA</t>
   </si>
   <si>
-    <t xml:space="preserve">For the Year Ended December 31, 2025</t>
+    <t xml:space="preserve">2025 Full Year + 2026 Year-to-Date (Jan-Mar Preliminary)</t>
   </si>
   <si>
     <t xml:space="preserve">Jan</t>
@@ -71,6 +71,18 @@
   </si>
   <si>
     <t xml:space="preserve">FY 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jan 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feb 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mar 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 YTD</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue</t>
@@ -944,11 +956,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:R105"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="15" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -968,6 +982,10 @@
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -986,6 +1004,10 @@
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
@@ -1004,6 +1026,10 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
@@ -1046,15 +1072,27 @@
       <c r="N5" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="O5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>492103</v>
@@ -1096,10 +1134,23 @@
         <f aca="false">SUM(B7:M7)</f>
         <v>6415025</v>
       </c>
+      <c r="O7" s="9" t="n">
+        <v>558871</v>
+      </c>
+      <c r="P7" s="9" t="n">
+        <v>569519</v>
+      </c>
+      <c r="Q7" s="9" t="n">
+        <v>570280</v>
+      </c>
+      <c r="R7" s="9" t="n">
+        <f aca="false">SUM(O7:Q7)</f>
+        <v>1698670</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>9897</v>
@@ -1141,10 +1192,23 @@
         <f aca="false">SUM(B8:M8)</f>
         <v>79101</v>
       </c>
+      <c r="O8" s="9" t="n">
+        <v>5055</v>
+      </c>
+      <c r="P8" s="9" t="n">
+        <v>5056</v>
+      </c>
+      <c r="Q8" s="9" t="n">
+        <v>4729</v>
+      </c>
+      <c r="R8" s="9" t="n">
+        <f aca="false">SUM(O8:Q8)</f>
+        <v>14840</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>13253</v>
@@ -1186,10 +1250,23 @@
         <f aca="false">SUM(B9:M9)</f>
         <v>119680</v>
       </c>
+      <c r="O9" s="9" t="n">
+        <v>8250</v>
+      </c>
+      <c r="P9" s="9" t="n">
+        <v>8249</v>
+      </c>
+      <c r="Q9" s="9" t="n">
+        <v>8256</v>
+      </c>
+      <c r="R9" s="9" t="n">
+        <f aca="false">SUM(O9:Q9)</f>
+        <v>24755</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>12039</v>
@@ -1231,10 +1308,23 @@
         <f aca="false">SUM(B10:M10)</f>
         <v>145426</v>
       </c>
+      <c r="O10" s="9" t="n">
+        <v>10551</v>
+      </c>
+      <c r="P10" s="9" t="n">
+        <v>10442</v>
+      </c>
+      <c r="Q10" s="9" t="n">
+        <v>10686</v>
+      </c>
+      <c r="R10" s="9" t="n">
+        <f aca="false">SUM(O10:Q10)</f>
+        <v>31679</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>10072</v>
@@ -1276,10 +1366,23 @@
         <f aca="false">SUM(B11:M11)</f>
         <v>94824</v>
       </c>
+      <c r="O11" s="9" t="n">
+        <v>4679</v>
+      </c>
+      <c r="P11" s="9" t="n">
+        <v>4352</v>
+      </c>
+      <c r="Q11" s="9" t="n">
+        <v>4346</v>
+      </c>
+      <c r="R11" s="9" t="n">
+        <f aca="false">SUM(O11:Q11)</f>
+        <v>13377</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">B7+B8+B9+B10+B11</f>
@@ -1333,10 +1436,26 @@
         <f aca="false">SUM(B12:M12)</f>
         <v>6854056</v>
       </c>
+      <c r="O12" s="11" t="n">
+        <f aca="false">O7+O8+O9+O10+O11</f>
+        <v>587406</v>
+      </c>
+      <c r="P12" s="11" t="n">
+        <f aca="false">P7+P8+P9+P10+P11</f>
+        <v>597618</v>
+      </c>
+      <c r="Q12" s="11" t="n">
+        <f aca="false">Q7+Q8+Q9+Q10+Q11</f>
+        <v>598297</v>
+      </c>
+      <c r="R12" s="11" t="n">
+        <f aca="false">R7+R8+R9+R10+R11</f>
+        <v>1783321</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B14" s="9" t="n">
         <v>1144</v>
@@ -1378,10 +1497,23 @@
         <f aca="false">SUM(B14:M14)</f>
         <v>13728</v>
       </c>
+      <c r="O14" s="9" t="n">
+        <v>1144</v>
+      </c>
+      <c r="P14" s="9" t="n">
+        <v>1144</v>
+      </c>
+      <c r="Q14" s="9" t="n">
+        <v>1144</v>
+      </c>
+      <c r="R14" s="9" t="n">
+        <f aca="false">SUM(O14:Q14)</f>
+        <v>3432</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>18993</v>
@@ -1423,10 +1555,23 @@
         <f aca="false">SUM(B15:M15)</f>
         <v>279518</v>
       </c>
+      <c r="O15" s="9" t="n">
+        <v>25891</v>
+      </c>
+      <c r="P15" s="9" t="n">
+        <v>25291</v>
+      </c>
+      <c r="Q15" s="9" t="n">
+        <v>25299</v>
+      </c>
+      <c r="R15" s="9" t="n">
+        <f aca="false">SUM(O15:Q15)</f>
+        <v>76481</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">B14+B15</f>
@@ -1480,10 +1625,26 @@
         <f aca="false">SUM(B16:M16)</f>
         <v>293246</v>
       </c>
+      <c r="O16" s="11" t="n">
+        <f aca="false">O14+O15</f>
+        <v>27035</v>
+      </c>
+      <c r="P16" s="11" t="n">
+        <f aca="false">P14+P15</f>
+        <v>26435</v>
+      </c>
+      <c r="Q16" s="11" t="n">
+        <f aca="false">Q14+Q15</f>
+        <v>26443</v>
+      </c>
+      <c r="R16" s="11" t="n">
+        <f aca="false">R14+R15</f>
+        <v>79913</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B18" s="9" t="n">
         <v>25121</v>
@@ -1525,10 +1686,23 @@
         <f aca="false">SUM(B18:M18)</f>
         <v>301506</v>
       </c>
+      <c r="O18" s="9" t="n">
+        <v>33254</v>
+      </c>
+      <c r="P18" s="9" t="n">
+        <v>33279</v>
+      </c>
+      <c r="Q18" s="9" t="n">
+        <v>33043</v>
+      </c>
+      <c r="R18" s="9" t="n">
+        <f aca="false">SUM(O18:Q18)</f>
+        <v>99576</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>562</v>
@@ -1570,10 +1744,23 @@
         <f aca="false">SUM(B19:M19)</f>
         <v>6749</v>
       </c>
+      <c r="O19" s="9" t="n">
+        <v>562</v>
+      </c>
+      <c r="P19" s="9" t="n">
+        <v>562</v>
+      </c>
+      <c r="Q19" s="9" t="n">
+        <v>562</v>
+      </c>
+      <c r="R19" s="9" t="n">
+        <f aca="false">SUM(O19:Q19)</f>
+        <v>1686</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>31136</v>
@@ -1615,10 +1802,23 @@
         <f aca="false">SUM(B20:M20)</f>
         <v>414530</v>
       </c>
+      <c r="O20" s="9" t="n">
+        <v>39621</v>
+      </c>
+      <c r="P20" s="9" t="n">
+        <v>39172</v>
+      </c>
+      <c r="Q20" s="9" t="n">
+        <v>39792</v>
+      </c>
+      <c r="R20" s="9" t="n">
+        <f aca="false">SUM(O20:Q20)</f>
+        <v>118585</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>974</v>
@@ -1660,10 +1860,23 @@
         <f aca="false">SUM(B21:M21)</f>
         <v>10927</v>
       </c>
+      <c r="O21" s="9" t="n">
+        <v>894</v>
+      </c>
+      <c r="P21" s="9" t="n">
+        <v>894</v>
+      </c>
+      <c r="Q21" s="9" t="n">
+        <v>891</v>
+      </c>
+      <c r="R21" s="9" t="n">
+        <f aca="false">SUM(O21:Q21)</f>
+        <v>2679</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>81227</v>
@@ -1705,10 +1918,23 @@
         <f aca="false">SUM(B22:M22)</f>
         <v>1156866</v>
       </c>
+      <c r="O22" s="9" t="n">
+        <v>125654</v>
+      </c>
+      <c r="P22" s="9" t="n">
+        <v>125038</v>
+      </c>
+      <c r="Q22" s="9" t="n">
+        <v>129650</v>
+      </c>
+      <c r="R22" s="9" t="n">
+        <f aca="false">SUM(O22:Q22)</f>
+        <v>380342</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>94782</v>
@@ -1750,10 +1976,23 @@
         <f aca="false">SUM(B23:M23)</f>
         <v>1526518</v>
       </c>
+      <c r="O23" s="9" t="n">
+        <v>157727</v>
+      </c>
+      <c r="P23" s="9" t="n">
+        <v>145432</v>
+      </c>
+      <c r="Q23" s="9" t="n">
+        <v>151908</v>
+      </c>
+      <c r="R23" s="9" t="n">
+        <f aca="false">SUM(O23:Q23)</f>
+        <v>455067</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B24" s="9" t="n">
         <v>4529</v>
@@ -1795,10 +2034,23 @@
         <f aca="false">SUM(B24:M24)</f>
         <v>47986</v>
       </c>
+      <c r="O24" s="9" t="n">
+        <v>5466</v>
+      </c>
+      <c r="P24" s="9" t="n">
+        <v>5166</v>
+      </c>
+      <c r="Q24" s="9" t="n">
+        <v>5166</v>
+      </c>
+      <c r="R24" s="9" t="n">
+        <f aca="false">SUM(O24:Q24)</f>
+        <v>15798</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B25" s="9" t="n">
         <v>641</v>
@@ -1840,10 +2092,23 @@
         <f aca="false">SUM(B25:M25)</f>
         <v>26687</v>
       </c>
+      <c r="O25" s="9" t="n">
+        <v>2546</v>
+      </c>
+      <c r="P25" s="9" t="n">
+        <v>2546</v>
+      </c>
+      <c r="Q25" s="9" t="n">
+        <v>2951</v>
+      </c>
+      <c r="R25" s="9" t="n">
+        <f aca="false">SUM(O25:Q25)</f>
+        <v>8043</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25</f>
@@ -1897,10 +2162,26 @@
         <f aca="false">SUM(B26:M26)</f>
         <v>3491769</v>
       </c>
+      <c r="O26" s="11" t="n">
+        <f aca="false">O18+O19+O20+O21+O22+O23+O24+O25</f>
+        <v>365724</v>
+      </c>
+      <c r="P26" s="11" t="n">
+        <f aca="false">P18+P19+P20+P21+P22+P23+P24+P25</f>
+        <v>352089</v>
+      </c>
+      <c r="Q26" s="11" t="n">
+        <f aca="false">Q18+Q19+Q20+Q21+Q22+Q23+Q24+Q25</f>
+        <v>363963</v>
+      </c>
+      <c r="R26" s="11" t="n">
+        <f aca="false">R18+R19+R20+R21+R22+R23+R24+R25</f>
+        <v>1081776</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B28" s="9" t="n">
         <v>51717</v>
@@ -1942,10 +2223,23 @@
         <f aca="false">SUM(B28:M28)</f>
         <v>940344</v>
       </c>
+      <c r="O28" s="9" t="n">
+        <v>24005</v>
+      </c>
+      <c r="P28" s="9" t="n">
+        <v>20890</v>
+      </c>
+      <c r="Q28" s="9" t="n">
+        <v>58595</v>
+      </c>
+      <c r="R28" s="9" t="n">
+        <f aca="false">SUM(O28:Q28)</f>
+        <v>103490</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B30" s="9" t="n">
         <v>86683</v>
@@ -1987,10 +2281,23 @@
         <f aca="false">SUM(B30:M30)</f>
         <v>320191</v>
       </c>
+      <c r="O30" s="9" t="n">
+        <v>36848</v>
+      </c>
+      <c r="P30" s="9" t="n">
+        <v>3570</v>
+      </c>
+      <c r="Q30" s="9" t="n">
+        <v>14827</v>
+      </c>
+      <c r="R30" s="9" t="n">
+        <f aca="false">SUM(O30:Q30)</f>
+        <v>55245</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B32" s="9" t="n">
         <v>203096</v>
@@ -2032,10 +2339,23 @@
         <f aca="false">SUM(B32:M32)</f>
         <v>5629784</v>
       </c>
+      <c r="O32" s="9" t="n">
+        <v>289324</v>
+      </c>
+      <c r="P32" s="9" t="n">
+        <v>236506</v>
+      </c>
+      <c r="Q32" s="9" t="n">
+        <v>357620</v>
+      </c>
+      <c r="R32" s="9" t="n">
+        <f aca="false">SUM(O32:Q32)</f>
+        <v>883450</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B33" s="9" t="n">
         <v>8709</v>
@@ -2077,10 +2397,23 @@
         <f aca="false">SUM(B33:M33)</f>
         <v>118378</v>
       </c>
+      <c r="O33" s="9" t="n">
+        <v>6435</v>
+      </c>
+      <c r="P33" s="9" t="n">
+        <v>7144</v>
+      </c>
+      <c r="Q33" s="9" t="n">
+        <v>8677</v>
+      </c>
+      <c r="R33" s="9" t="n">
+        <f aca="false">SUM(O33:Q33)</f>
+        <v>22256</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">B32+B33</f>
@@ -2134,10 +2467,26 @@
         <f aca="false">SUM(B34:M34)</f>
         <v>5748162</v>
       </c>
+      <c r="O34" s="11" t="n">
+        <f aca="false">O32+O33</f>
+        <v>295759</v>
+      </c>
+      <c r="P34" s="11" t="n">
+        <f aca="false">P32+P33</f>
+        <v>243650</v>
+      </c>
+      <c r="Q34" s="11" t="n">
+        <f aca="false">Q32+Q33</f>
+        <v>366297</v>
+      </c>
+      <c r="R34" s="11" t="n">
+        <f aca="false">R32+R33</f>
+        <v>905706</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B36" s="9" t="n">
         <v>5590</v>
@@ -2179,10 +2528,23 @@
         <f aca="false">SUM(B36:M36)</f>
         <v>89645</v>
       </c>
+      <c r="O36" s="9" t="n">
+        <v>15537</v>
+      </c>
+      <c r="P36" s="9" t="n">
+        <v>12379</v>
+      </c>
+      <c r="Q36" s="9" t="n">
+        <v>11648</v>
+      </c>
+      <c r="R36" s="9" t="n">
+        <f aca="false">SUM(O36:Q36)</f>
+        <v>39564</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B38" s="13" t="n">
         <f aca="false">B12+B16+B26+B28+B30+B34+B36</f>
@@ -2236,15 +2598,31 @@
         <f aca="false">SUM(B38:M38)</f>
         <v>17737413</v>
       </c>
+      <c r="O38" s="13" t="n">
+        <f aca="false">O12+O16+O26+O28+O30+O34+O36</f>
+        <v>1352314</v>
+      </c>
+      <c r="P38" s="13" t="n">
+        <f aca="false">P12+P16+P26+P28+P30+P34+P36</f>
+        <v>1256631</v>
+      </c>
+      <c r="Q38" s="13" t="n">
+        <f aca="false">Q12+Q16+Q26+Q28+Q30+Q34+Q36</f>
+        <v>1440070</v>
+      </c>
+      <c r="R38" s="13" t="n">
+        <f aca="false">R12+R16+R26+R28+R30+R34+R36</f>
+        <v>4049015</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B42" s="9" t="n">
         <v>22885</v>
@@ -2286,10 +2664,23 @@
         <f aca="false">SUM(B42:M42)</f>
         <v>308646</v>
       </c>
+      <c r="O42" s="9" t="n">
+        <v>133469</v>
+      </c>
+      <c r="P42" s="9" t="n">
+        <v>191612</v>
+      </c>
+      <c r="Q42" s="9" t="n">
+        <v>24897</v>
+      </c>
+      <c r="R42" s="9" t="n">
+        <f aca="false">SUM(O42:Q42)</f>
+        <v>349978</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B43" s="9" t="n">
         <v>8915</v>
@@ -2331,10 +2722,23 @@
         <f aca="false">SUM(B43:M43)</f>
         <v>130837</v>
       </c>
+      <c r="O43" s="9" t="n">
+        <v>11555</v>
+      </c>
+      <c r="P43" s="9" t="n">
+        <v>9883</v>
+      </c>
+      <c r="Q43" s="9" t="n">
+        <v>12306</v>
+      </c>
+      <c r="R43" s="9" t="n">
+        <f aca="false">SUM(O43:Q43)</f>
+        <v>33744</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B44" s="9" t="n">
         <v>157949</v>
@@ -2376,10 +2780,23 @@
         <f aca="false">SUM(B44:M44)</f>
         <v>2209537</v>
       </c>
+      <c r="O44" s="9" t="n">
+        <v>152678</v>
+      </c>
+      <c r="P44" s="9" t="n">
+        <v>162239</v>
+      </c>
+      <c r="Q44" s="9" t="n">
+        <v>224409</v>
+      </c>
+      <c r="R44" s="9" t="n">
+        <f aca="false">SUM(O44:Q44)</f>
+        <v>539326</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B45" s="9" t="n">
         <v>0</v>
@@ -2421,10 +2838,23 @@
         <f aca="false">SUM(B45:M45)</f>
         <v>2899</v>
       </c>
+      <c r="O45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="R45" s="9" t="n">
+        <f aca="false">SUM(O45:Q45)</f>
+        <v>8</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B46" s="9" t="n">
         <v>72436</v>
@@ -2466,10 +2896,23 @@
         <f aca="false">SUM(B46:M46)</f>
         <v>290943</v>
       </c>
+      <c r="O46" s="9" t="n">
+        <v>30947</v>
+      </c>
+      <c r="P46" s="9" t="n">
+        <v>2975</v>
+      </c>
+      <c r="Q46" s="9" t="n">
+        <v>13392</v>
+      </c>
+      <c r="R46" s="9" t="n">
+        <f aca="false">SUM(O46:Q46)</f>
+        <v>47314</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B47" s="9" t="n">
         <v>180392</v>
@@ -2511,10 +2954,23 @@
         <f aca="false">SUM(B47:M47)</f>
         <v>4891735</v>
       </c>
+      <c r="O47" s="9" t="n">
+        <v>251712</v>
+      </c>
+      <c r="P47" s="9" t="n">
+        <v>205760</v>
+      </c>
+      <c r="Q47" s="9" t="n">
+        <v>318110</v>
+      </c>
+      <c r="R47" s="9" t="n">
+        <f aca="false">SUM(O47:Q47)</f>
+        <v>775582</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B48" s="9" t="n">
         <v>69884</v>
@@ -2556,10 +3012,23 @@
         <f aca="false">SUM(B48:M48)</f>
         <v>761019</v>
       </c>
+      <c r="O48" s="9" t="n">
+        <v>60926</v>
+      </c>
+      <c r="P48" s="9" t="n">
+        <v>49371</v>
+      </c>
+      <c r="Q48" s="9" t="n">
+        <v>57301</v>
+      </c>
+      <c r="R48" s="9" t="n">
+        <f aca="false">SUM(O48:Q48)</f>
+        <v>167598</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B49" s="9" t="n">
         <v>227678</v>
@@ -2601,10 +3070,23 @@
         <f aca="false">SUM(B49:M49)</f>
         <v>2496470</v>
       </c>
+      <c r="O49" s="9" t="n">
+        <v>226198</v>
+      </c>
+      <c r="P49" s="9" t="n">
+        <v>134465</v>
+      </c>
+      <c r="Q49" s="9" t="n">
+        <v>151433</v>
+      </c>
+      <c r="R49" s="9" t="n">
+        <f aca="false">SUM(O49:Q49)</f>
+        <v>512096</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B50" s="13" t="n">
         <f aca="false">B42+B43+B44+B45+B46+B47+B48+B49</f>
@@ -2658,10 +3140,26 @@
         <f aca="false">SUM(B50:M50)</f>
         <v>11092086</v>
       </c>
+      <c r="O50" s="13" t="n">
+        <f aca="false">O42+O43+O44+O45+O46+O47+O48+O49</f>
+        <v>867485</v>
+      </c>
+      <c r="P50" s="13" t="n">
+        <f aca="false">P42+P43+P44+P45+P46+P47+P48+P49</f>
+        <v>756305</v>
+      </c>
+      <c r="Q50" s="13" t="n">
+        <f aca="false">Q42+Q43+Q44+Q45+Q46+Q47+Q48+Q49</f>
+        <v>801856</v>
+      </c>
+      <c r="R50" s="13" t="n">
+        <f aca="false">R42+R43+R44+R45+R46+R47+R48+R49</f>
+        <v>2425646</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B52" s="13" t="n">
         <f aca="false">B38-B50</f>
@@ -2715,10 +3213,26 @@
         <f aca="false">SUM(B52:M52)</f>
         <v>6645327</v>
       </c>
+      <c r="O52" s="13" t="n">
+        <f aca="false">O38-O50</f>
+        <v>484829</v>
+      </c>
+      <c r="P52" s="13" t="n">
+        <f aca="false">P38-P50</f>
+        <v>500326</v>
+      </c>
+      <c r="Q52" s="13" t="n">
+        <f aca="false">Q38-Q50</f>
+        <v>638214</v>
+      </c>
+      <c r="R52" s="13" t="n">
+        <f aca="false">R38-R50</f>
+        <v>1623369</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B53" s="15" t="n">
         <f aca="false">IF(B38=0,0,B52/B38)</f>
@@ -2772,10 +3286,26 @@
         <f aca="false">IF(N38=0,0,N52/N38)</f>
         <v>0.374650294267828</v>
       </c>
+      <c r="O53" s="15" t="n">
+        <f aca="false">IF(O38=0,0,O52/O38)</f>
+        <v>0.358518066070454</v>
+      </c>
+      <c r="P53" s="15" t="n">
+        <f aca="false">IF(P38=0,0,P52/P38)</f>
+        <v>0.398148700772144</v>
+      </c>
+      <c r="Q53" s="15" t="n">
+        <f aca="false">IF(Q38=0,0,Q52/Q38)</f>
+        <v>0.443182623066934</v>
+      </c>
+      <c r="R53" s="15" t="n">
+        <f aca="false">IF(R38=0,0,R52/R38)</f>
+        <v>0.400929361832446</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B55" s="9" t="n">
         <v>174805</v>
@@ -2817,15 +3347,28 @@
         <f aca="false">SUM(B55:M55)</f>
         <v>1757071</v>
       </c>
+      <c r="O55" s="9" t="n">
+        <v>128659</v>
+      </c>
+      <c r="P55" s="9" t="n">
+        <v>114856</v>
+      </c>
+      <c r="Q55" s="9" t="n">
+        <v>134018</v>
+      </c>
+      <c r="R55" s="9" t="n">
+        <f aca="false">SUM(O55:Q55)</f>
+        <v>377533</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B59" s="9" t="n">
         <v>88384</v>
@@ -2867,10 +3410,23 @@
         <f aca="false">SUM(B59:M59)</f>
         <v>974855</v>
       </c>
+      <c r="O59" s="9" t="n">
+        <v>70635</v>
+      </c>
+      <c r="P59" s="9" t="n">
+        <v>33491</v>
+      </c>
+      <c r="Q59" s="9" t="n">
+        <v>57494</v>
+      </c>
+      <c r="R59" s="9" t="n">
+        <f aca="false">SUM(O59:Q59)</f>
+        <v>161620</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B60" s="9" t="n">
         <v>26216</v>
@@ -2912,10 +3468,23 @@
         <f aca="false">SUM(B60:M60)</f>
         <v>308929</v>
       </c>
+      <c r="O60" s="9" t="n">
+        <v>21807</v>
+      </c>
+      <c r="P60" s="9" t="n">
+        <v>21807</v>
+      </c>
+      <c r="Q60" s="9" t="n">
+        <v>21807</v>
+      </c>
+      <c r="R60" s="9" t="n">
+        <f aca="false">SUM(O60:Q60)</f>
+        <v>65421</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B61" s="9" t="n">
         <v>299</v>
@@ -2957,10 +3526,23 @@
         <f aca="false">SUM(B61:M61)</f>
         <v>27718</v>
       </c>
+      <c r="O61" s="9" t="n">
+        <v>781</v>
+      </c>
+      <c r="P61" s="9" t="n">
+        <v>3701</v>
+      </c>
+      <c r="Q61" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" s="9" t="n">
+        <f aca="false">SUM(O61:Q61)</f>
+        <v>4482</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B62" s="9" t="n">
         <v>13535</v>
@@ -3002,10 +3584,23 @@
         <f aca="false">SUM(B62:M62)</f>
         <v>160771</v>
       </c>
+      <c r="O62" s="9" t="n">
+        <v>14080</v>
+      </c>
+      <c r="P62" s="9" t="n">
+        <v>12269</v>
+      </c>
+      <c r="Q62" s="9" t="n">
+        <v>14704</v>
+      </c>
+      <c r="R62" s="9" t="n">
+        <f aca="false">SUM(O62:Q62)</f>
+        <v>41053</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B63" s="9" t="n">
         <v>27164</v>
@@ -3047,10 +3642,23 @@
         <f aca="false">SUM(B63:M63)</f>
         <v>414606</v>
       </c>
+      <c r="O63" s="9" t="n">
+        <v>54781</v>
+      </c>
+      <c r="P63" s="9" t="n">
+        <v>14333</v>
+      </c>
+      <c r="Q63" s="9" t="n">
+        <v>99702</v>
+      </c>
+      <c r="R63" s="9" t="n">
+        <f aca="false">SUM(O63:Q63)</f>
+        <v>168816</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B64" s="9" t="n">
         <v>55295</v>
@@ -3092,10 +3700,23 @@
         <f aca="false">SUM(B64:M64)</f>
         <v>713009</v>
       </c>
+      <c r="O64" s="9" t="n">
+        <v>59667</v>
+      </c>
+      <c r="P64" s="9" t="n">
+        <v>71792</v>
+      </c>
+      <c r="Q64" s="9" t="n">
+        <v>75806</v>
+      </c>
+      <c r="R64" s="9" t="n">
+        <f aca="false">SUM(O64:Q64)</f>
+        <v>207265</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B65" s="9" t="n">
         <v>0</v>
@@ -3137,10 +3758,23 @@
         <f aca="false">SUM(B65:M65)</f>
         <v>0</v>
       </c>
+      <c r="O65" s="9" t="n">
+        <v>-12431</v>
+      </c>
+      <c r="P65" s="9" t="n">
+        <v>47924</v>
+      </c>
+      <c r="Q65" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" s="9" t="n">
+        <f aca="false">SUM(O65:Q65)</f>
+        <v>35493</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="8" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B66" s="9" t="n">
         <v>6971</v>
@@ -3182,10 +3816,23 @@
         <f aca="false">SUM(B66:M66)</f>
         <v>79909</v>
       </c>
+      <c r="O66" s="9" t="n">
+        <v>8102</v>
+      </c>
+      <c r="P66" s="9" t="n">
+        <v>7431</v>
+      </c>
+      <c r="Q66" s="9" t="n">
+        <v>8718</v>
+      </c>
+      <c r="R66" s="9" t="n">
+        <f aca="false">SUM(O66:Q66)</f>
+        <v>24251</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B67" s="9" t="n">
         <v>4520</v>
@@ -3227,10 +3874,23 @@
         <f aca="false">SUM(B67:M67)</f>
         <v>114962</v>
       </c>
+      <c r="O67" s="9" t="n">
+        <v>20060</v>
+      </c>
+      <c r="P67" s="9" t="n">
+        <v>8685</v>
+      </c>
+      <c r="Q67" s="9" t="n">
+        <v>119</v>
+      </c>
+      <c r="R67" s="9" t="n">
+        <f aca="false">SUM(O67:Q67)</f>
+        <v>28864</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B68" s="9" t="n">
         <v>7654</v>
@@ -3272,10 +3932,23 @@
         <f aca="false">SUM(B68:M68)</f>
         <v>104423</v>
       </c>
+      <c r="O68" s="9" t="n">
+        <v>10459</v>
+      </c>
+      <c r="P68" s="9" t="n">
+        <v>10975</v>
+      </c>
+      <c r="Q68" s="9" t="n">
+        <v>17821</v>
+      </c>
+      <c r="R68" s="9" t="n">
+        <f aca="false">SUM(O68:Q68)</f>
+        <v>39255</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="8" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B69" s="9" t="n">
         <v>285</v>
@@ -3317,10 +3990,23 @@
         <f aca="false">SUM(B69:M69)</f>
         <v>17984</v>
       </c>
+      <c r="O69" s="9" t="n">
+        <v>5287</v>
+      </c>
+      <c r="P69" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="Q69" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="R69" s="9" t="n">
+        <f aca="false">SUM(O69:Q69)</f>
+        <v>15332</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="8" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B70" s="9" t="n">
         <v>4179</v>
@@ -3362,10 +4048,23 @@
         <f aca="false">SUM(B70:M70)</f>
         <v>37733</v>
       </c>
+      <c r="O70" s="9" t="n">
+        <v>16493</v>
+      </c>
+      <c r="P70" s="9" t="n">
+        <v>2018</v>
+      </c>
+      <c r="Q70" s="9" t="n">
+        <v>1930</v>
+      </c>
+      <c r="R70" s="9" t="n">
+        <f aca="false">SUM(O70:Q70)</f>
+        <v>20441</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="8" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B71" s="9" t="n">
         <v>6399</v>
@@ -3407,10 +4106,23 @@
         <f aca="false">SUM(B71:M71)</f>
         <v>78398</v>
       </c>
+      <c r="O71" s="9" t="n">
+        <v>5678</v>
+      </c>
+      <c r="P71" s="9" t="n">
+        <v>40609</v>
+      </c>
+      <c r="Q71" s="9" t="n">
+        <v>21933</v>
+      </c>
+      <c r="R71" s="9" t="n">
+        <f aca="false">SUM(O71:Q71)</f>
+        <v>68220</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="8" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B72" s="9" t="n">
         <v>1688</v>
@@ -3452,10 +4164,23 @@
         <f aca="false">SUM(B72:M72)</f>
         <v>31221</v>
       </c>
+      <c r="O72" s="9" t="n">
+        <v>8513</v>
+      </c>
+      <c r="P72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R72" s="9" t="n">
+        <f aca="false">SUM(O72:Q72)</f>
+        <v>8513</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B73" s="9" t="n">
         <v>7425</v>
@@ -3497,10 +4222,23 @@
         <f aca="false">SUM(B73:M73)</f>
         <v>228578</v>
       </c>
+      <c r="O73" s="9" t="n">
+        <v>11195</v>
+      </c>
+      <c r="P73" s="9" t="n">
+        <v>2967</v>
+      </c>
+      <c r="Q73" s="9" t="n">
+        <v>10335</v>
+      </c>
+      <c r="R73" s="9" t="n">
+        <f aca="false">SUM(O73:Q73)</f>
+        <v>24497</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B74" s="13" t="n">
         <f aca="false">B59+B60+B61+B62+B63+B64+B65+B66+B67+B68+B69+B70+B71+B72+B73</f>
@@ -3554,10 +4292,26 @@
         <f aca="false">SUM(B74:M74)</f>
         <v>3293096</v>
       </c>
+      <c r="O74" s="13" t="n">
+        <f aca="false">SUM(O59:O73)</f>
+        <v>295107</v>
+      </c>
+      <c r="P74" s="13" t="n">
+        <f aca="false">SUM(P59:P73)</f>
+        <v>288002</v>
+      </c>
+      <c r="Q74" s="13" t="n">
+        <f aca="false">SUM(Q59:Q73)</f>
+        <v>330414</v>
+      </c>
+      <c r="R74" s="13" t="n">
+        <f aca="false">SUM(R59:R73)</f>
+        <v>913523</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="16" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B77" s="17" t="n">
         <f aca="false">B52-B55-B74</f>
@@ -3611,10 +4365,26 @@
         <f aca="false">SUM(B77:M77)</f>
         <v>1595160</v>
       </c>
+      <c r="O77" s="17" t="n">
+        <f aca="false">O52-O55-O74</f>
+        <v>61063</v>
+      </c>
+      <c r="P77" s="17" t="n">
+        <f aca="false">P52-P55-P74</f>
+        <v>97468</v>
+      </c>
+      <c r="Q77" s="17" t="n">
+        <f aca="false">Q52-Q55-Q74</f>
+        <v>173782</v>
+      </c>
+      <c r="R77" s="17" t="n">
+        <f aca="false">R52-R55-R74</f>
+        <v>332313</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="14" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B78" s="15" t="n">
         <f aca="false">IF(B38=0,0,B77/B38)</f>
@@ -3668,10 +4438,26 @@
         <f aca="false">IF(N38=0,0,N77/N38)</f>
         <v>0.0899319421609002</v>
       </c>
+      <c r="O78" s="15" t="n">
+        <f aca="false">IF(O38=0,0,O77/O38)</f>
+        <v>0.04515445377331</v>
+      </c>
+      <c r="P78" s="15" t="n">
+        <f aca="false">IF(P38=0,0,P77/P38)</f>
+        <v>0.0775629440941693</v>
+      </c>
+      <c r="Q78" s="15" t="n">
+        <f aca="false">IF(Q38=0,0,Q77/Q38)</f>
+        <v>0.120676078246196</v>
+      </c>
+      <c r="R78" s="15" t="n">
+        <f aca="false">IF(R38=0,0,R77/R38)</f>
+        <v>0.0820725534481843</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="18" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B80" s="19"/>
       <c r="C80" s="19"/>
@@ -3686,10 +4472,14 @@
       <c r="L80" s="19"/>
       <c r="M80" s="19"/>
       <c r="N80" s="19"/>
+      <c r="O80" s="19"/>
+      <c r="P80" s="19"/>
+      <c r="Q80" s="19"/>
+      <c r="R80" s="19"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B81" s="21" t="s">
         <v>3</v>
@@ -3728,12 +4518,24 @@
         <v>14</v>
       </c>
       <c r="N81" s="21" t="s">
-        <v>76</v>
+        <v>80</v>
+      </c>
+      <c r="O81" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="P81" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q81" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="R81" s="21" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="22" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B82" s="23" t="n">
         <v>15700</v>
@@ -3775,10 +4577,23 @@
         <f aca="false">SUM(B82:M82)</f>
         <v>188400</v>
       </c>
+      <c r="O82" s="23" t="n">
+        <v>15700</v>
+      </c>
+      <c r="P82" s="23" t="n">
+        <v>15700</v>
+      </c>
+      <c r="Q82" s="23" t="n">
+        <v>15700</v>
+      </c>
+      <c r="R82" s="24" t="n">
+        <f aca="false">SUM(O82:Q82)</f>
+        <v>47100</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="25" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B83" s="26"/>
       <c r="C83" s="26"/>
@@ -3806,10 +4621,23 @@
         <f aca="false">SUM(B83:M83)</f>
         <v>20000</v>
       </c>
+      <c r="O83" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="P83" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="Q83" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="R83" s="27" t="n">
+        <f aca="false">SUM(O83:Q83)</f>
+        <v>12000</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B84" s="23" t="n">
         <v>12750</v>
@@ -3851,10 +4679,23 @@
         <f aca="false">SUM(B84:M84)</f>
         <v>153000</v>
       </c>
+      <c r="O84" s="23" t="n">
+        <v>12750</v>
+      </c>
+      <c r="P84" s="23" t="n">
+        <v>12750</v>
+      </c>
+      <c r="Q84" s="23" t="n">
+        <v>12750</v>
+      </c>
+      <c r="R84" s="24" t="n">
+        <f aca="false">SUM(O84:Q84)</f>
+        <v>38250</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="25" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B85" s="26"/>
       <c r="C85" s="26"/>
@@ -3876,10 +4717,14 @@
         <f aca="false">SUM(B85:M85)</f>
         <v>10888</v>
       </c>
+      <c r="R85" s="27" t="n">
+        <f aca="false">SUM(O85:Q85)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="22" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B86" s="23"/>
       <c r="C86" s="23"/>
@@ -3911,10 +4756,14 @@
         <f aca="false">SUM(B86:M86)</f>
         <v>42000</v>
       </c>
+      <c r="R86" s="24" t="n">
+        <f aca="false">SUM(O86:Q86)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B87" s="26" t="n">
         <v>3520</v>
@@ -3956,10 +4805,23 @@
         <f aca="false">SUM(B87:M87)</f>
         <v>42240</v>
       </c>
+      <c r="O87" s="26" t="n">
+        <v>3520</v>
+      </c>
+      <c r="P87" s="26" t="n">
+        <v>3520</v>
+      </c>
+      <c r="Q87" s="26" t="n">
+        <v>3520</v>
+      </c>
+      <c r="R87" s="27" t="n">
+        <f aca="false">SUM(O87:Q87)</f>
+        <v>10560</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B88" s="23" t="n">
         <v>12000</v>
@@ -4001,10 +4863,23 @@
         <f aca="false">SUM(B88:M88)</f>
         <v>115960</v>
       </c>
+      <c r="O88" s="23" t="n">
+        <v>8000</v>
+      </c>
+      <c r="P88" s="23" t="n">
+        <v>8000</v>
+      </c>
+      <c r="Q88" s="23" t="n">
+        <v>8000</v>
+      </c>
+      <c r="R88" s="24" t="n">
+        <f aca="false">SUM(O88:Q88)</f>
+        <v>24000</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B89" s="26"/>
       <c r="C89" s="26"/>
@@ -4024,10 +4899,14 @@
         <f aca="false">SUM(B89:M89)</f>
         <v>231000</v>
       </c>
+      <c r="R89" s="27" t="n">
+        <f aca="false">SUM(O89:Q89)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="22" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B90" s="23"/>
       <c r="C90" s="23"/>
@@ -4047,10 +4926,14 @@
         <f aca="false">SUM(B90:M90)</f>
         <v>70940</v>
       </c>
+      <c r="R90" s="24" t="n">
+        <f aca="false">SUM(O90:Q90)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="25" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B91" s="26" t="n">
         <v>25000</v>
@@ -4070,10 +4953,14 @@
         <f aca="false">SUM(B91:M91)</f>
         <v>25000</v>
       </c>
+      <c r="R91" s="27" t="n">
+        <f aca="false">SUM(O91:Q91)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="22" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B92" s="23" t="n">
         <v>8500</v>
@@ -4095,10 +4982,14 @@
         <f aca="false">SUM(B92:M92)</f>
         <v>17000</v>
       </c>
+      <c r="R92" s="24" t="n">
+        <f aca="false">SUM(O92:Q92)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="25" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B93" s="26" t="n">
         <v>8000</v>
@@ -4128,10 +5019,14 @@
         <f aca="false">SUM(B93:M93)</f>
         <v>48000</v>
       </c>
+      <c r="R93" s="27" t="n">
+        <f aca="false">SUM(O93:Q93)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="22" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B94" s="23"/>
       <c r="C94" s="23"/>
@@ -4153,10 +5048,14 @@
         <f aca="false">SUM(B94:M94)</f>
         <v>30000</v>
       </c>
+      <c r="R94" s="24" t="n">
+        <f aca="false">SUM(O94:Q94)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B95" s="26"/>
       <c r="C95" s="26" t="n">
@@ -4176,10 +5075,14 @@
         <f aca="false">SUM(B95:M95)</f>
         <v>10000</v>
       </c>
+      <c r="R95" s="27" t="n">
+        <f aca="false">SUM(O95:Q95)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="22" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B96" s="23"/>
       <c r="C96" s="23"/>
@@ -4199,10 +5102,14 @@
         <f aca="false">SUM(B96:M96)</f>
         <v>20000</v>
       </c>
+      <c r="R96" s="24" t="n">
+        <f aca="false">SUM(O96:Q96)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="25" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B97" s="26"/>
       <c r="C97" s="26"/>
@@ -4222,10 +5129,14 @@
         <f aca="false">SUM(B97:M97)</f>
         <v>20000</v>
       </c>
+      <c r="R97" s="27" t="n">
+        <f aca="false">SUM(O97:Q97)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="22" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B98" s="23" t="n">
         <v>6174</v>
@@ -4261,10 +5172,14 @@
         <f aca="false">SUM(B98:M98)</f>
         <v>55566</v>
       </c>
+      <c r="R98" s="24" t="n">
+        <f aca="false">SUM(O98:Q98)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="25" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B99" s="26" t="n">
         <v>5167</v>
@@ -4306,10 +5221,23 @@
         <f aca="false">SUM(B99:M99)</f>
         <v>62000</v>
       </c>
+      <c r="O99" s="26" t="n">
+        <v>5167</v>
+      </c>
+      <c r="P99" s="26" t="n">
+        <v>5167</v>
+      </c>
+      <c r="Q99" s="26" t="n">
+        <v>5167</v>
+      </c>
+      <c r="R99" s="27" t="n">
+        <f aca="false">SUM(O99:Q99)</f>
+        <v>15501</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="22" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B100" s="23"/>
       <c r="C100" s="23"/>
@@ -4329,10 +5257,14 @@
         <f aca="false">SUM(B100:M100)</f>
         <v>135253</v>
       </c>
+      <c r="R100" s="24" t="n">
+        <f aca="false">SUM(O100:Q100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="28" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B101" s="29" t="n">
         <f aca="false">SUM(B84:B100)</f>
@@ -4385,6 +5317,22 @@
       <c r="N101" s="29" t="n">
         <f aca="false">SUM(N82:N100)</f>
         <v>1297247</v>
+      </c>
+      <c r="O101" s="29" t="n">
+        <f aca="false">SUM(O84:O100)</f>
+        <v>29437</v>
+      </c>
+      <c r="P101" s="29" t="n">
+        <f aca="false">SUM(P84:P100)</f>
+        <v>29437</v>
+      </c>
+      <c r="Q101" s="29" t="n">
+        <f aca="false">SUM(Q84:Q100)</f>
+        <v>29437</v>
+      </c>
+      <c r="R101" s="29" t="n">
+        <f aca="false">SUM(R82:R100)</f>
+        <v>147411</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4405,7 +5353,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="31" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B103" s="32" t="n">
         <f aca="false">B77+B101</f>
@@ -4459,10 +5407,26 @@
         <f aca="false">N77+N101</f>
         <v>2892407</v>
       </c>
+      <c r="O103" s="32" t="n">
+        <f aca="false">O77+O101</f>
+        <v>90500</v>
+      </c>
+      <c r="P103" s="32" t="n">
+        <f aca="false">P77+P101</f>
+        <v>126905</v>
+      </c>
+      <c r="Q103" s="32" t="n">
+        <f aca="false">Q77+Q101</f>
+        <v>203219</v>
+      </c>
+      <c r="R103" s="32" t="n">
+        <f aca="false">R77+R101</f>
+        <v>479724</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="33" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B104" s="34" t="n">
         <f aca="false">IF(B38=0,0,B103/B38)</f>
@@ -4515,6 +5479,22 @@
       <c r="N104" s="34" t="n">
         <f aca="false">IF(N38=0,0,N103/N38)</f>
         <v>0.163068143026269</v>
+      </c>
+      <c r="O104" s="34" t="n">
+        <f aca="false">IF(O38=0,0,O103/O38)</f>
+        <v>0.066922327210988</v>
+      </c>
+      <c r="P104" s="34" t="n">
+        <f aca="false">IF(P38=0,0,P103/P38)</f>
+        <v>0.100988277386122</v>
+      </c>
+      <c r="Q104" s="34" t="n">
+        <f aca="false">IF(Q38=0,0,Q103/Q38)</f>
+        <v>0.141117445679724</v>
+      </c>
+      <c r="R104" s="34" t="n">
+        <f aca="false">IF(R38=0,0,R103/R38)</f>
+        <v>0.118479185678492</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4535,9 +5515,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A3:R3"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>